<commit_message>
Set target performance level (75) for each mapped program learning outcome
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y7qFGHCWANDz1tZ3jcQYcG
</commit_message>
<xml_diff>
--- a/نواتج_التعلم_التصميم_الجرافيكي_2025-2026.xlsx
+++ b/نواتج_التعلم_التصميم_الجرافيكي_2025-2026.xlsx
@@ -3476,19 +3476,25 @@
           <t>يتعرف على المفاهيم والنظريات والاتجاهات الفنية في مجال التصميم الجرافيكي.</t>
         </is>
       </c>
-      <c r="C3" s="46"/>
+      <c r="C3" s="46">
+        <v>75</v>
+      </c>
       <c r="D3" s="39" t="inlineStr">
         <is>
           <t>يستعرض خصائص الخامات الرقمية والأدوات والتطبيقات التقنية وطرق استخدامها.</t>
         </is>
       </c>
-      <c r="E3" s="46"/>
+      <c r="E3" s="46">
+        <v>75</v>
+      </c>
       <c r="F3" s="39" t="inlineStr">
         <is>
           <t>يوضح الأساليب الفنية والتقنية والبحثية المختلفة في مجال التصميم الجرافيكي.</t>
         </is>
       </c>
-      <c r="G3" s="46"/>
+      <c r="G3" s="46">
+        <v>75</v>
+      </c>
       <c r="H3" s="39"/>
       <c r="I3" s="46"/>
       <c r="K3" s="46"/>
@@ -3497,22 +3503,33 @@
           <t>يقارن بين الأدوات والأساليب التقنية والمعرفية في مجال التصميم الجرافيكي.</t>
         </is>
       </c>
-      <c r="M3" s="46"/>
+      <c r="M3" s="46">
+        <v>75</v>
+      </c>
       <c r="N3" s="39"/>
       <c r="R3" s="39" t="inlineStr">
         <is>
           <t>يتعاون بفاعلية ضمن مجموعات العمل من خلال العروض التقديمية والكتابية لبناء العلاقات المهنية.</t>
         </is>
       </c>
+      <c r="S3" s="46">
+        <v>75</v>
+      </c>
       <c r="V3" s="39" t="inlineStr">
         <is>
           <t>يطبق المفاهيم والمهارات والاستراتيجيات والنظريات في مجال التصميم الجرافيكي.</t>
         </is>
       </c>
+      <c r="W3" s="46">
+        <v>75</v>
+      </c>
       <c r="X3" s="39" t="inlineStr">
         <is>
           <t>يصمم باستخدام التقنيات والبرامج لإنتاج أعمال تساهم في تعزيز الهوية الوطنية والثقافية.</t>
         </is>
+      </c>
+      <c r="Y3" s="46">
+        <v>75</v>
       </c>
       <c r="Z3" s="46"/>
       <c r="AB3" s="39" t="inlineStr">
@@ -3520,17 +3537,25 @@
           <t>ينتج أعمالاً وتقارير ومشاريع مبتكرة في مجال التصميم الجرافيكي تساهم في الرفع من جودة الحياة.</t>
         </is>
       </c>
-      <c r="AC3" s="46"/>
+      <c r="AC3" s="46">
+        <v>75</v>
+      </c>
       <c r="AE3" s="46"/>
       <c r="AJ3" s="39" t="inlineStr">
         <is>
           <t>يلتزم بالأخلاقيات المهنية والحقوق الفكرية في التصميم.</t>
         </is>
       </c>
+      <c r="AK3" s="46">
+        <v>75</v>
+      </c>
       <c r="AL3" s="39" t="inlineStr">
         <is>
           <t>يقدر أهمية العمل اليدوي والتقني وارتباطه بالهوية الثقافية.</t>
         </is>
+      </c>
+      <c r="AM3" s="46">
+        <v>75</v>
       </c>
       <c r="AR3" s="43"/>
       <c r="AS3" s="43"/>

</xml_diff>